<commit_message>
Added Table and documents related to C7
</commit_message>
<xml_diff>
--- a/C7/C7 tables.xlsx
+++ b/C7/C7 tables.xlsx
@@ -129,9 +129,6 @@
     <t xml:space="preserve">2. Students are from rural area, mostly educated in local language medium, weak in understanding. </t>
   </si>
   <si>
-    <t>3. Students weak in CNC programming.</t>
-  </si>
-  <si>
     <r>
       <t>Action 1:</t>
     </r>
@@ -336,11 +333,8 @@
     <t>PO5</t>
   </si>
   <si>
-    <t xml:space="preserve">1. The courses of mechanical Engineering are addressing the needs of, health, safety and social concerns regarding engineering practices in real life. </t>
-  </si>
-  <si>
-    <r>
-      <t>Action: 1.</t>
+    <r>
+      <t xml:space="preserve">Action: 2. </t>
     </r>
     <r>
       <rPr>
@@ -349,35 +343,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve"> Environmental studies course incorporated in MSBTE curriculum to aware the students regarding Importance of Environmental Studies, Natural Resources, Ecosystems, Biodiversity and its Conservation, Environmental Pollution, Social Issues and Environment, Environmental Protection.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Action: 2. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
       <t>Participation of students in cleanliness drive and tree plantation.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Action: 3. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Expert lecture on personality development and health awareness arranged.</t>
     </r>
   </si>
   <si>
@@ -707,6 +673,9 @@
     </r>
   </si>
   <si>
+    <t>3. Students were weak in hadling/opearting computer</t>
+  </si>
+  <si>
     <r>
       <t>Action 3:</t>
     </r>
@@ -717,7 +686,38 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve"> CNC programming practical arranged to be familiar with the CNC coding.</t>
+      <t xml:space="preserve"> Extra sessions are arranged in Fudamental of ICT subject.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Action: 1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Subjects like Social and Life Skills, Essence Of Indian Constitution, Environmental Education And Sustainability are incorporated in MSBTE curriculum to aware the students regarding Importance of Environmental Studies, Natural Resources, Ecosystems, Biodiversity and its Conservation, Environmental Pollution, Social Issues and Environment, Environmental Protection.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The courses of Computer Engineering Programs are addressing the needs of health, safety and social concerns regarding engineering practices in real life. </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Action: 3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Expert lecture on Yoga and Meditation, Personality development and health awareness arranged.</t>
     </r>
   </si>
 </sst>
@@ -775,7 +775,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -806,8 +806,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="30">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -846,50 +858,6 @@
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
@@ -957,19 +925,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top/>
       <bottom style="medium">
@@ -992,133 +947,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -1156,208 +984,115 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1639,7 +1374,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
@@ -1649,631 +1384,577 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="62" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="62" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="59">
-        <v>2.4700000000000002</v>
-      </c>
-      <c r="C3" s="59">
-        <v>2.14</v>
-      </c>
-      <c r="D3" s="60" t="s">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="51"/>
+      <c r="E3" s="15"/>
     </row>
     <row r="4" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58"/>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="60" t="s">
+      <c r="A4" s="13"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="51"/>
+      <c r="E4" s="15"/>
     </row>
     <row r="5" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58"/>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="60" t="s">
+      <c r="A5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="51"/>
+      <c r="E5" s="15"/>
     </row>
     <row r="6" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="61"/>
-      <c r="C6" s="61"/>
-      <c r="D6" s="61"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="61"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="61"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="63" t="s">
+      <c r="A8" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="63"/>
-      <c r="C8" s="63"/>
-      <c r="D8" s="63"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="54" t="s">
+      <c r="A9" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="56">
-        <v>1.84</v>
-      </c>
-      <c r="C9" s="64">
-        <v>1.72</v>
-      </c>
-      <c r="D9" s="57" t="s">
+      <c r="B9" s="18"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="51"/>
+      <c r="E9" s="15"/>
     </row>
     <row r="10" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="54"/>
-      <c r="B10" s="56"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="57" t="s">
+      <c r="A10" s="17"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="51"/>
+      <c r="E10" s="15"/>
     </row>
     <row r="11" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="54"/>
-      <c r="B11" s="56"/>
-      <c r="C11" s="64"/>
-      <c r="D11" s="57" t="s">
+      <c r="A11" s="17"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="15"/>
+    </row>
+    <row r="12" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="51"/>
-    </row>
-    <row r="12" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="55" t="s">
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="55" t="s">
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="55"/>
-      <c r="C13" s="55"/>
-      <c r="D13" s="55"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="55" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="65" t="s">
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="65"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="65"/>
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="54" t="s">
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="64">
-        <v>1.85</v>
-      </c>
-      <c r="C16" s="64">
-        <v>1.72</v>
-      </c>
-      <c r="D16" s="57" t="s">
+      <c r="E16" s="15"/>
+    </row>
+    <row r="17" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="17"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="51"/>
-    </row>
-    <row r="17" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="54"/>
-      <c r="B17" s="64"/>
-      <c r="C17" s="64"/>
-      <c r="D17" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="E17" s="51"/>
+      <c r="E17" s="15"/>
     </row>
     <row r="18" spans="1:5" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="1:5" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="19" t="s">
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="65" t="s">
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="65"/>
-      <c r="C20" s="65"/>
-      <c r="D20" s="65"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="54" t="s">
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="64">
-        <v>1.9</v>
-      </c>
-      <c r="C21" s="64">
-        <v>1.76</v>
-      </c>
-      <c r="D21" s="57" t="s">
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="17"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="54"/>
-      <c r="B22" s="64"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="57" t="s">
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="55" t="s">
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="55"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55"/>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="55" t="s">
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="55"/>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="1"/>
-    </row>
-    <row r="25" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="63" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="63"/>
-      <c r="C25" s="63"/>
-      <c r="D25" s="63"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
       <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="1:5" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="15"/>
+    </row>
+    <row r="28" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="15"/>
+    </row>
+    <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="15"/>
+    </row>
+    <row r="30" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="15"/>
+    </row>
+    <row r="31" spans="1:5" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="15"/>
+    </row>
+    <row r="32" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" spans="1:5" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="28"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="15"/>
+    </row>
+    <row r="35" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="15"/>
+    </row>
+    <row r="36" spans="1:5" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="15"/>
+    </row>
+    <row r="37" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="15"/>
+    </row>
+    <row r="38" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="1"/>
+    </row>
+    <row r="39" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E39" s="1"/>
+    </row>
+    <row r="40" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="15"/>
+    </row>
+    <row r="41" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="15"/>
+    </row>
+    <row r="42" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="15"/>
+    </row>
+    <row r="43" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" s="30"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
+      <c r="E43" s="1"/>
+    </row>
+    <row r="44" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" s="11">
+        <v>1.58</v>
+      </c>
+      <c r="C44" s="11">
+        <v>1.65</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E44" s="1"/>
+    </row>
+    <row r="45" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="B45" s="32"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="1"/>
+    </row>
+    <row r="46" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46" s="30"/>
+      <c r="C46" s="30"/>
+      <c r="D46" s="30"/>
+      <c r="E46" s="1"/>
+    </row>
+    <row r="47" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A47" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47" s="11">
+        <v>1.87</v>
+      </c>
+      <c r="C47" s="11">
         <v>1.76</v>
       </c>
-      <c r="C26" s="11">
-        <v>1.68</v>
-      </c>
-      <c r="D26" s="66" t="s">
-        <v>32</v>
-      </c>
-      <c r="E26" s="1"/>
-    </row>
-    <row r="27" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="55" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="55"/>
-      <c r="C27" s="55"/>
-      <c r="D27" s="55"/>
-      <c r="E27" s="51"/>
-    </row>
-    <row r="28" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="55" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" s="55"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="51"/>
-    </row>
-    <row r="29" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="55" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="55"/>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="51"/>
-    </row>
-    <row r="30" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="55" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="55"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="51"/>
-    </row>
-    <row r="31" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="67" t="s">
-        <v>37</v>
-      </c>
-      <c r="B31" s="67"/>
-      <c r="C31" s="67"/>
-      <c r="D31" s="67"/>
-      <c r="E31" s="51"/>
-    </row>
-    <row r="32" spans="1:5" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="63" t="s">
-        <v>38</v>
-      </c>
-      <c r="B32" s="63"/>
-      <c r="C32" s="63"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="1"/>
-    </row>
-    <row r="33" spans="1:5" ht="48" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="5">
-        <v>1.85</v>
-      </c>
-      <c r="C33" s="5">
-        <v>1.76</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="30"/>
-      <c r="B34" s="31"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="18"/>
-    </row>
-    <row r="35" spans="1:5" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="33"/>
-      <c r="C35" s="33"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="18"/>
-    </row>
-    <row r="36" spans="1:5" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="B36" s="33"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="18"/>
-    </row>
-    <row r="37" spans="1:5" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33"/>
-      <c r="D37" s="34"/>
-      <c r="E37" s="18"/>
-    </row>
-    <row r="38" spans="1:5" ht="110.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="18"/>
-    </row>
-    <row r="39" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="1"/>
-    </row>
-    <row r="40" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="14"/>
-      <c r="B40" s="35"/>
-      <c r="C40" s="35"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="1"/>
-    </row>
-    <row r="41" spans="1:5" ht="378.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B41" s="5">
-        <v>1.9</v>
-      </c>
-      <c r="C41" s="5">
-        <v>1.77</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E41" s="1"/>
-    </row>
-    <row r="42" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="18"/>
-    </row>
-    <row r="43" spans="1:5" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="B43" s="33"/>
-      <c r="C43" s="33"/>
-      <c r="D43" s="34"/>
-      <c r="E43" s="18"/>
-    </row>
-    <row r="44" spans="1:5" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="B44" s="28"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="18"/>
-    </row>
-    <row r="45" spans="1:5" ht="94.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="1"/>
-    </row>
-    <row r="46" spans="1:5" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B46" s="5">
-        <v>1.58</v>
-      </c>
-      <c r="C46" s="5">
+      <c r="D47" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E47" s="1"/>
+    </row>
+    <row r="48" spans="1:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="1"/>
+    </row>
+    <row r="49" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B49" s="34"/>
+      <c r="C49" s="34"/>
+      <c r="D49" s="34"/>
+      <c r="E49" s="1"/>
+    </row>
+    <row r="50" spans="1:5" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50" s="30"/>
+      <c r="C50" s="30"/>
+      <c r="D50" s="30"/>
+      <c r="E50" s="1"/>
+    </row>
+    <row r="51" spans="1:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B51" s="35">
+        <v>1.71</v>
+      </c>
+      <c r="C51" s="35">
         <v>1.65</v>
       </c>
-      <c r="D46" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E46" s="1"/>
-    </row>
-    <row r="47" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="B47" s="38"/>
-      <c r="C47" s="38"/>
-      <c r="D47" s="39"/>
-      <c r="E47" s="1"/>
-    </row>
-    <row r="48" spans="1:5" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B48" s="41"/>
-      <c r="C48" s="41"/>
-      <c r="D48" s="42"/>
-      <c r="E48" s="1"/>
-    </row>
-    <row r="49" spans="1:5" ht="174" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B49" s="9">
-        <v>1.87</v>
-      </c>
-      <c r="C49" s="9">
-        <v>1.76</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E49" s="1"/>
-    </row>
-    <row r="50" spans="1:5" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="19" t="s">
+      <c r="D51" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="21"/>
-      <c r="E50" s="1"/>
-    </row>
-    <row r="51" spans="1:5" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="43" t="s">
+      <c r="E51" s="1"/>
+    </row>
+    <row r="52" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B51" s="44"/>
-      <c r="C51" s="44"/>
-      <c r="D51" s="45"/>
-      <c r="E51" s="1"/>
-    </row>
-    <row r="52" spans="1:5" ht="94.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="46" t="s">
+      <c r="B52" s="28"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="15"/>
+    </row>
+    <row r="53" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B52" s="47"/>
-      <c r="C52" s="47"/>
-      <c r="D52" s="48"/>
-      <c r="E52" s="1"/>
-    </row>
-    <row r="53" spans="1:5" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="B53" s="12">
-        <v>1.71</v>
-      </c>
-      <c r="C53" s="12">
-        <v>1.65</v>
-      </c>
-      <c r="D53" s="49" t="s">
-        <v>62</v>
-      </c>
-      <c r="E53" s="1"/>
-    </row>
-    <row r="54" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="13"/>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="50"/>
-      <c r="E54" s="1"/>
-    </row>
-    <row r="55" spans="1:5" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="B55" s="31"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="32"/>
-      <c r="E55" s="18"/>
-    </row>
-    <row r="56" spans="1:5" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="B56" s="28"/>
-      <c r="C56" s="28"/>
-      <c r="D56" s="29"/>
-      <c r="E56" s="18"/>
+      <c r="B53" s="28"/>
+      <c r="C53" s="28"/>
+      <c r="D53" s="28"/>
+      <c r="E53" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="60">
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="E55:E56"/>
+  <mergeCells count="55">
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A49:D49"/>
     <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="E42:E44"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A36:D36"/>
     <mergeCell ref="A37:D37"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="E40:E42"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A45:D45"/>
     <mergeCell ref="A38:D38"/>
-    <mergeCell ref="E34:E38"/>
-    <mergeCell ref="A39:D40"/>
-    <mergeCell ref="A42:D42"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="E27:E31"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="A18:D18"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="A21:A22"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="C21:C22"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="E9:E11"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="A14:D14"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="E3:E5"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="B9:B11"/>
     <mergeCell ref="C9:C11"/>
-    <mergeCell ref="E9:E11"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="C3:C5"/>
+    <mergeCell ref="E3:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Added PO1-3 gap analysis in Report and Sheet
</commit_message>
<xml_diff>
--- a/C7/C7 tables.xlsx
+++ b/C7/C7 tables.xlsx
@@ -50,43 +50,6 @@
     <t>PO1</t>
   </si>
   <si>
-    <t>1. At entry level the students are observed weak in basic fundamental subjects.</t>
-  </si>
-  <si>
-    <t>2. Students are weak in their soft skills and unable to grasp engineering fundamentals.</t>
-  </si>
-  <si>
-    <t>3. Tutorial sessions were not adequate looking towards entry level of students.</t>
-  </si>
-  <si>
-    <r>
-      <t>Action 1:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Tutorial sessions arranged for mathematical subjects.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Action 2:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Expert lectures arranged for courses and in the curriculum of MSBTE core technical subjects .</t>
-    </r>
-  </si>
-  <si>
     <r>
       <t>PO2</t>
     </r>
@@ -130,34 +93,6 @@
   </si>
   <si>
     <r>
-      <t>Action 1:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">  Extra lectures are arranged to enhance the basic knowledge.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Action 2:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Tutorial session   arranged and assignments are given for more practice.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">PO3 </t>
     </r>
     <r>
@@ -191,40 +126,6 @@
   </si>
   <si>
     <t>PO3</t>
-  </si>
-  <si>
-    <t>1. Performance in prerequisite courses is poor.</t>
-  </si>
-  <si>
-    <t>2. Students weak in numerical courses.</t>
-  </si>
-  <si>
-    <r>
-      <t>Action 1:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">  Extra lectures conducted for SOM, DME and TEN.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Action 2:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Industry visit arranged to enhance design and development concepts.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -673,23 +574,6 @@
     </r>
   </si>
   <si>
-    <t>3. Students were weak in hadling/opearting computer</t>
-  </si>
-  <si>
-    <r>
-      <t>Action 3:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Extra sessions are arranged in Fudamental of ICT subject.</t>
-    </r>
-  </si>
-  <si>
     <r>
       <t>Action: 1.</t>
     </r>
@@ -718,6 +602,122 @@
         <family val="1"/>
       </rPr>
       <t>Expert lecture on Yoga and Meditation, Personality development and health awareness arranged.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Action 3: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Bilingual notes/Lab manuals were made available to students on MSBTE website to overcome language barriers.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Action 1:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Weak students pertaining to basic discipline knowledge were identified by conducting baseline test for first year students.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Action 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> E-contents were made availabe to students for grasping the concepts easily</t>
+    </r>
+  </si>
+  <si>
+    <t>1. At entry level the students were observed weak in basic fundamental subjects.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Students were weak in their soft skills and unable to grasp engineering fundamentals </t>
+  </si>
+  <si>
+    <t>3. Tutorial sessions were not adequate looking towards entry level of students. Extra practice / contents were needed.</t>
+  </si>
+  <si>
+    <t>3. Students are weak in hadling/opearting computer</t>
+  </si>
+  <si>
+    <r>
+      <t>Action 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Tutorial sessions are arranged and assignments were given for more practice.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Action 1:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  Extra lectures are arranged to enhance the basic knowledge as well as handling of computers.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Students struggle to design ER Diagram i.e Scheme design rather than just SQL Commands. </t>
+  </si>
+  <si>
+    <t>2. Students had theoretical knowledge of topologies but couldn't design a functional small-scale network.</t>
+  </si>
+  <si>
+    <r>
+      <t>Action 1:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Implemented mandatory ER Diagram before actully going to SQL Commands. Students must present their ER Diagram to the instructor for approval.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Action 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Students are asked to form group of four and asked to search and demostrate animation of actual packet transfer on Internet</t>
     </r>
   </si>
 </sst>
@@ -775,7 +775,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -815,6 +815,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -984,7 +990,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1019,8 +1025,74 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1028,71 +1100,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1366,7 +1384,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1399,400 +1417,400 @@
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="18"/>
+    </row>
+    <row r="4" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="35"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="18"/>
+    </row>
+    <row r="5" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="35"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="18"/>
+    </row>
+    <row r="6" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="15"/>
-    </row>
-    <row r="4" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="8" t="s">
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="15"/>
-    </row>
-    <row r="5" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="8" t="s">
+      <c r="B10" s="34"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="15"/>
-    </row>
-    <row r="6" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="E10" s="18"/>
+    </row>
+    <row r="11" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="28"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+      <c r="E11" s="18"/>
+    </row>
+    <row r="12" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="28"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="18"/>
+    </row>
+    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="18"/>
+    </row>
+    <row r="17" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="37"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" s="18"/>
+    </row>
+    <row r="18" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="7" t="s">
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="15"/>
-    </row>
-    <row r="10" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="7" t="s">
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="15"/>
-    </row>
-    <row r="11" spans="1:5" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E11" s="15"/>
-    </row>
-    <row r="12" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="28"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="20" t="s">
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="15"/>
-    </row>
-    <row r="17" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="15"/>
-    </row>
-    <row r="18" spans="1:5" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="1:5" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="17"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="1"/>
-    </row>
-    <row r="25" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
       <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
-      <c r="D26" s="29" t="s">
-        <v>64</v>
+      <c r="D26" s="12" t="s">
+        <v>51</v>
       </c>
       <c r="E26" s="1"/>
     </row>
     <row r="27" spans="1:5" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="15"/>
+      <c r="A27" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="18"/>
     </row>
     <row r="28" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="15"/>
+      <c r="A28" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="18"/>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="15"/>
+      <c r="A29" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="18"/>
     </row>
     <row r="30" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="15"/>
+      <c r="A30" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="18"/>
     </row>
     <row r="31" spans="1:5" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="15"/>
+      <c r="A31" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="18"/>
     </row>
     <row r="32" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
+      <c r="A32" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
       <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:5" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="5" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="E33" s="1"/>
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="28"/>
-      <c r="C34" s="28"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="15"/>
+      <c r="A34" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="18"/>
     </row>
     <row r="35" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="15"/>
+      <c r="A35" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="18"/>
     </row>
     <row r="36" spans="1:5" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" s="28"/>
-      <c r="C36" s="28"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="15"/>
+      <c r="A36" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="18"/>
     </row>
     <row r="37" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="15"/>
+      <c r="A37" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="18"/>
     </row>
     <row r="38" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
+      <c r="A38" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="23"/>
       <c r="E38" s="1"/>
     </row>
     <row r="39" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
       <c r="D39" s="10" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E39" s="1"/>
     </row>
     <row r="40" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="B40" s="28"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="15"/>
+      <c r="A40" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="18"/>
     </row>
     <row r="41" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="15"/>
+      <c r="A41" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="18"/>
     </row>
     <row r="42" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="B42" s="28"/>
-      <c r="C42" s="28"/>
-      <c r="D42" s="28"/>
-      <c r="E42" s="15"/>
+      <c r="A42" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="18"/>
     </row>
     <row r="43" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="B43" s="30"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
+      <c r="A43" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
       <c r="E43" s="1"/>
     </row>
     <row r="44" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="31" t="s">
-        <v>48</v>
+      <c r="A44" s="13" t="s">
+        <v>37</v>
       </c>
       <c r="B44" s="11">
         <v>1.58</v>
@@ -1801,31 +1819,31 @@
         <v>1.65</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E44" s="1"/>
     </row>
     <row r="45" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="B45" s="32"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="32"/>
+      <c r="A45" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
       <c r="E45" s="1"/>
     </row>
     <row r="46" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="B46" s="30"/>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
+      <c r="A46" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
       <c r="E46" s="1"/>
     </row>
     <row r="47" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="33" t="s">
-        <v>52</v>
+      <c r="A47" s="14" t="s">
+        <v>41</v>
       </c>
       <c r="B47" s="11">
         <v>1.87</v>
@@ -1834,78 +1852,108 @@
         <v>1.76</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E47" s="1"/>
     </row>
     <row r="48" spans="1:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
+      <c r="A48" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B48" s="19"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
       <c r="E48" s="1"/>
     </row>
     <row r="49" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B49" s="34"/>
-      <c r="C49" s="34"/>
-      <c r="D49" s="34"/>
+      <c r="A49" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B49" s="20"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="20"/>
       <c r="E49" s="1"/>
     </row>
     <row r="50" spans="1:5" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="B50" s="30"/>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
+      <c r="A50" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B50" s="21"/>
+      <c r="C50" s="21"/>
+      <c r="D50" s="21"/>
       <c r="E50" s="1"/>
     </row>
     <row r="51" spans="1:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="35" t="s">
-        <v>57</v>
-      </c>
-      <c r="B51" s="35">
+      <c r="A51" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B51" s="15">
         <v>1.71</v>
       </c>
-      <c r="C51" s="35">
+      <c r="C51" s="15">
         <v>1.65</v>
       </c>
-      <c r="D51" s="36" t="s">
-        <v>58</v>
+      <c r="D51" s="16" t="s">
+        <v>47</v>
       </c>
       <c r="E51" s="1"/>
     </row>
     <row r="52" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="B52" s="28"/>
-      <c r="C52" s="28"/>
-      <c r="D52" s="28"/>
-      <c r="E52" s="15"/>
+      <c r="A52" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="18"/>
     </row>
     <row r="53" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="B53" s="28"/>
-      <c r="C53" s="28"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="15"/>
+      <c r="A53" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="55">
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="E27:E31"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="A46:D46"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A36:D36"/>
@@ -1919,42 +1967,12 @@
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="E27:E31"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="E9:E11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A50:D50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Made Changes in C6 as per suggetions from Lalbondre Sir
</commit_message>
<xml_diff>
--- a/C7/C7 tables.xlsx
+++ b/C7/C7 tables.xlsx
@@ -1040,77 +1040,77 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1384,7 +1384,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1417,227 +1417,227 @@
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
       <c r="D3" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="18"/>
+      <c r="E3" s="22"/>
     </row>
     <row r="4" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="35"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
       <c r="D4" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="18"/>
+      <c r="E4" s="22"/>
     </row>
     <row r="5" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="35"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E5" s="18"/>
+      <c r="E5" s="22"/>
     </row>
     <row r="6" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="29"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="26"/>
       <c r="D10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="22"/>
     </row>
     <row r="11" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28"/>
-      <c r="B11" s="34"/>
-      <c r="C11" s="29"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="26"/>
       <c r="D11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="22"/>
     </row>
     <row r="12" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="29"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="26"/>
       <c r="D12" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="22"/>
     </row>
     <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="39" t="s">
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="18"/>
+      <c r="E16" s="22"/>
     </row>
     <row r="17" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="37"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="40" t="s">
+      <c r="A17" s="29"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="18"/>
+      <c r="E17" s="22"/>
     </row>
     <row r="18" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="33"/>
       <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="26"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="36"/>
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
       <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
       <c r="D21" s="7" t="s">
         <v>14</v>
       </c>
       <c r="E21" s="1"/>
     </row>
     <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
       <c r="D22" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
       <c r="E23" s="1"/>
     </row>
     <row r="24" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
       <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
@@ -1652,57 +1652,57 @@
       <c r="E26" s="1"/>
     </row>
     <row r="27" spans="1:5" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="18"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="18"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="22"/>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="18"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="22"/>
     </row>
     <row r="30" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="18"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="22"/>
     </row>
     <row r="31" spans="1:5" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="18"/>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="22"/>
     </row>
     <row r="32" spans="1:5" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="23" t="s">
+      <c r="A32" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
       <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:5" ht="48" thickBot="1" x14ac:dyDescent="0.3">
@@ -1717,48 +1717,48 @@
       <c r="E33" s="1"/>
     </row>
     <row r="34" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="18"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="22"/>
     </row>
     <row r="35" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="18"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="22"/>
     </row>
     <row r="36" spans="1:5" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="18"/>
+      <c r="B36" s="37"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="22"/>
     </row>
     <row r="37" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="18"/>
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="22"/>
     </row>
     <row r="38" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="23" t="s">
+      <c r="A38" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="1"/>
     </row>
     <row r="39" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
@@ -1773,39 +1773,39 @@
       <c r="E39" s="1"/>
     </row>
     <row r="40" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="18"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="37"/>
+      <c r="E40" s="22"/>
     </row>
     <row r="41" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="17" t="s">
+      <c r="A41" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="18"/>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+      <c r="E41" s="22"/>
     </row>
     <row r="42" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="18"/>
+      <c r="B42" s="37"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="37"/>
+      <c r="E42" s="22"/>
     </row>
     <row r="43" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B43" s="21"/>
-      <c r="C43" s="21"/>
-      <c r="D43" s="21"/>
+      <c r="B43" s="38"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
       <c r="E43" s="1"/>
     </row>
     <row r="44" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -1824,21 +1824,21 @@
       <c r="E44" s="1"/>
     </row>
     <row r="45" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="22" t="s">
+      <c r="A45" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
+      <c r="B45" s="39"/>
+      <c r="C45" s="39"/>
+      <c r="D45" s="39"/>
       <c r="E45" s="1"/>
     </row>
     <row r="46" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B46" s="21"/>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
+      <c r="B46" s="38"/>
+      <c r="C46" s="38"/>
+      <c r="D46" s="38"/>
       <c r="E46" s="1"/>
     </row>
     <row r="47" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -1857,30 +1857,30 @@
       <c r="E47" s="1"/>
     </row>
     <row r="48" spans="1:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="B48" s="19"/>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
+      <c r="B48" s="27"/>
+      <c r="C48" s="27"/>
+      <c r="D48" s="27"/>
       <c r="E48" s="1"/>
     </row>
     <row r="49" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="20" t="s">
+      <c r="A49" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
+      <c r="B49" s="40"/>
+      <c r="C49" s="40"/>
+      <c r="D49" s="40"/>
       <c r="E49" s="1"/>
     </row>
     <row r="50" spans="1:5" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="21" t="s">
+      <c r="A50" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="B50" s="21"/>
-      <c r="C50" s="21"/>
-      <c r="D50" s="21"/>
+      <c r="B50" s="38"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="38"/>
       <c r="E50" s="1"/>
     </row>
     <row r="51" spans="1:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1899,61 +1899,31 @@
       <c r="E51" s="1"/>
     </row>
     <row r="52" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="17" t="s">
+      <c r="A52" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="B52" s="17"/>
-      <c r="C52" s="17"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="18"/>
+      <c r="B52" s="37"/>
+      <c r="C52" s="37"/>
+      <c r="D52" s="37"/>
+      <c r="E52" s="22"/>
     </row>
     <row r="53" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="17" t="s">
+      <c r="A53" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="18"/>
+      <c r="B53" s="37"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
+      <c r="E53" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="55">
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="E27:E31"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A50:D50"/>
     <mergeCell ref="A46:D46"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A36:D36"/>
@@ -1967,12 +1937,42 @@
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="E27:E31"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="E3:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>